<commit_message>
Assign a size from the same voucher to previously unspecified-size rows
</commit_message>
<xml_diff>
--- a/vouchers_1404.xlsx
+++ b/vouchers_1404.xlsx
@@ -457,7 +457,7 @@
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
   </cols>
@@ -4694,7 +4694,11 @@
           <t>نامشخص ⚠</t>
         </is>
       </c>
-      <c r="N81" s="2" t="inlineStr"/>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>44 (تخمینی)⚠</t>
+        </is>
+      </c>
       <c r="O81" s="2" t="n">
         <v>1</v>
       </c>
@@ -4742,7 +4746,11 @@
           <t>نامشخص ⚠</t>
         </is>
       </c>
-      <c r="N82" s="2" t="inlineStr"/>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>44 (تخمینی)⚠</t>
+        </is>
+      </c>
       <c r="O82" s="2" t="n">
         <v>1</v>
       </c>
@@ -4790,7 +4798,11 @@
           <t>نامشخص ⚠</t>
         </is>
       </c>
-      <c r="N83" s="2" t="inlineStr"/>
+      <c r="N83" s="2" t="inlineStr">
+        <is>
+          <t>44 (تخمینی)⚠</t>
+        </is>
+      </c>
       <c r="O83" s="2" t="n">
         <v>1</v>
       </c>
@@ -5098,7 +5110,11 @@
           <t>نامشخص ⚠</t>
         </is>
       </c>
-      <c r="N89" s="2" t="inlineStr"/>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>XXXL (تخمینی)⚠</t>
+        </is>
+      </c>
       <c r="O89" s="2" t="n">
         <v>1</v>
       </c>

</xml_diff>